<commit_message>
Update ArchingCoefficients -> ArchingCoefficient references for diggs-schema PB1 rename
diggs-schema renamed ArchingCoefficients/ArchingCoefficientsType (and the archingCoefficients
property) to their singular forms. The conditionalElementXpath (ri_design_properties.xlsx, 10
entries) and sourceElementXpath (archingModel.xlsx, 7 entries) values that reference the element
by name are functional, not prose, so the source workbooks were edited and both dictionaries
regenerated via dict_xml_convert.py --only.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/archingModel.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/archingModel.xlsx
@@ -1679,7 +1679,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>//diggs:ArchingCoefficients/diggs:archingModel</t>
+          <t>//diggs:ArchingCoefficient/diggs:archingModel</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1695,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>//diggs:ArchingCoefficients/diggs:archingModel</t>
+          <t>//diggs:ArchingCoefficient/diggs:archingModel</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>//diggs:ArchingCoefficients/diggs:archingModel</t>
+          <t>//diggs:ArchingCoefficient/diggs:archingModel</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>//diggs:ArchingCoefficients/diggs:archingModel</t>
+          <t>//diggs:ArchingCoefficient/diggs:archingModel</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>//diggs:ArchingCoefficients/diggs:archingModel</t>
+          <t>//diggs:ArchingCoefficient/diggs:archingModel</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>//diggs:ArchingCoefficients/diggs:archingModel</t>
+          <t>//diggs:ArchingCoefficient/diggs:archingModel</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>//diggs:ArchingCoefficients/diggs:archingModel</t>
+          <t>//diggs:ArchingCoefficient/diggs:archingModel</t>
         </is>
       </c>
     </row>

</xml_diff>